<commit_message>
Minor bugfixes for src
</commit_message>
<xml_diff>
--- a/data/Fig1/Sup1/Cqresults.xlsx
+++ b/data/Fig1/Sup1/Cqresults.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\PHD_data\Imaging_et_analysis\PaperFigures\Figure1\Sup\QpCR\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\snaik\Desktop\Paperpublishgit\data\Fig1\Sup1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C7C7B28-5E48-4B58-9AC2-480C658CBD06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28020" yWindow="780" windowWidth="21600" windowHeight="12645" xr2:uid="{FBD0258E-EA1C-49B5-A8FF-833AB2442DF3}"/>
+    <workbookView xWindow="-28020" yWindow="780" windowWidth="21600" windowHeight="12645"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateCount="1"/>
+  <calcPr calcId="162913" iterateCount="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -96,7 +95,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.00_);\(0.00\)"/>
     <numFmt numFmtId="165" formatCode="0.00_ ;\-0.00\ "/>
@@ -182,7 +181,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{983F8C5D-CEE1-4A85-82D8-4A7B92C7D586}"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -493,7 +492,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB8ED0B4-2D25-498C-9998-2D0A73EC1FB2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -734,22 +733,22 @@
         <v>-4.4931977294227181</v>
       </c>
       <c r="D9">
-        <v>-6.9338551850976877</v>
+        <v>-5.9338551850976904</v>
       </c>
       <c r="E9" s="12">
         <v>-5.1839621838381333</v>
       </c>
       <c r="F9" s="1">
         <f t="shared" si="0"/>
-        <v>-5.4308439020648933</v>
+        <v>-5.1808439020648942</v>
       </c>
       <c r="G9">
         <f t="shared" si="1"/>
-        <v>0.45418921689321945</v>
+        <v>0.2555121021849574</v>
       </c>
       <c r="H9" s="3">
         <f t="shared" si="2"/>
-        <v>43.136699822038324</v>
+        <v>36.273496246227609</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>